<commit_message>
feat(fields): add IMB/PTECH required fields per v2.0 + BOM global items (project mgmt/warehouse/survey/as-built), TC-01 fixture updated
</commit_message>
<xml_diff>
--- a/tests/data/regression/TC-01_正确工程案例.xlsx
+++ b/tests/data/regression/TC-01_正确工程案例.xlsx
@@ -694,7 +694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -708,6 +708,21 @@
           <t>归属节点</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>QUARTIER</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>NOM_VOIE</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>NOM_BATIMENT</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -720,6 +735,21 @@
           <t>BPE-TNG01-BOK01-002</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>QUARTIER-1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>NOM_VOIE-1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>NOM_BATIMENT-1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -730,6 +760,21 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>BPE-TNG01-BOK01-003</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>QUARTIER-1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NOM_VOIE-1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NOM_BATIMENT-1</t>
         </is>
       </c>
     </row>
@@ -794,7 +839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,6 +853,11 @@
           <t>类型</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>NOM</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -820,6 +870,11 @@
           <t>技术点</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>NOM-1</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -830,6 +885,11 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>技术点</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NOM-1</t>
         </is>
       </c>
     </row>

</xml_diff>